<commit_message>
dayOfWeek and template fixes
</commit_message>
<xml_diff>
--- a/backend/Scheduler/Export/template.xlsx
+++ b/backend/Scheduler/Export/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\военка\Desktop\Sheduler\schedule\backend\Scheduler\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB522675-F549-4C81-908D-A7F44B7D3478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{288D1C29-A58C-4A80-8797-5E733755F9BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="874" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">взвод!$A$1:$T$22</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">подвал!$A$1:$T$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">подвал!$A$1:$T$10</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">шапка!$A$1:$T$4</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>08.30-10.00</t>
   </si>
@@ -62,46 +62,28 @@
     <t>12.00-12.40</t>
   </si>
   <si>
-    <t>СРЕДА</t>
-  </si>
-  <si>
     <t>15.15-16.45</t>
   </si>
   <si>
     <t>дата</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">РАСПИСАНИЕ ЗАНЯТИЙ
-с гражданами, проходящими военную подготовку по ВУС </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="48"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="48"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-        <charset val="204"/>
-      </rPr>
-      <t xml:space="preserve">в  семестре  учебного года    </t>
-    </r>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>ЧЕТВЕРГ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">РАСПИСАНИЕ ЗАНЯТИЙ
+с гражданами, проходящими военную подготовку по ВУС 
+в  семестре  учебного года </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,19 +184,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="24"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
-      <sz val="48"/>
-      <color rgb="FFFF0000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-      <charset val="204"/>
-    </font>
-    <font>
       <sz val="26"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -237,7 +206,6 @@
     <font>
       <b/>
       <sz val="48"/>
-      <color rgb="FFFF0000"/>
       <name val="Courier New"/>
       <family val="3"/>
       <charset val="204"/>
@@ -804,12 +772,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="49" fontId="11" fillId="2" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -825,21 +787,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -981,22 +928,46 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1065,14 +1036,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" shrinkToFit="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1113,17 +1081,17 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>1835492</xdr:colOff>
+      <xdr:colOff>1841494</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>150813</xdr:rowOff>
+      <xdr:rowOff>158750</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="9483991" cy="3238500"/>
+    <xdr:ext cx="9493250" cy="3238500"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="TextBox 1">
+        <xdr:cNvPr id="3" name="TextBox 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{68193E66-3F2F-4BE2-9F92-3ED36F6819F6}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{28703DD9-AD4E-4EB5-A757-1A34B9409A34}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1131,8 +1099,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="47771392" y="150813"/>
-          <a:ext cx="9483991" cy="3238500"/>
+          <a:off x="47777394" y="158750"/>
+          <a:ext cx="9493250" cy="3238500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1231,34 +1199,14 @@
               <a:latin typeface="Times New Roman" pitchFamily="18" charset="0"/>
               <a:cs typeface="Times New Roman" pitchFamily="18" charset="0"/>
             </a:rPr>
-            <a:t>июля  202</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="3400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman" pitchFamily="18" charset="0"/>
-              <a:cs typeface="Times New Roman" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t>5</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="ru-RU" sz="3400">
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-              <a:latin typeface="Times New Roman" pitchFamily="18" charset="0"/>
-              <a:cs typeface="Times New Roman" pitchFamily="18" charset="0"/>
-            </a:rPr>
-            <a:t> </a:t>
+            <a:t>июля 2025 </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="ru-RU" sz="3400">
               <a:latin typeface="Times New Roman" pitchFamily="18" charset="0"/>
               <a:cs typeface="Times New Roman" pitchFamily="18" charset="0"/>
             </a:rPr>
-            <a:t>года</a:t>
+            <a:t>года </a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -1273,22 +1221,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>895805</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:colOff>246064</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>285749</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>942150</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>191827</xdr:rowOff>
+      <xdr:colOff>1190626</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>215636</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
+        <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{402DBD8C-15A9-411B-ABB3-2771252B2CDC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73119FA6-8015-426C-A1A9-797974B88203}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1296,8 +1244,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16986705" y="15827375"/>
-          <a:ext cx="23922345" cy="1357052"/>
+          <a:off x="16336964" y="37661849"/>
+          <a:ext cx="24820562" cy="1580887"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1656,102 +1604,106 @@
   <dimension ref="A1:T4"/>
   <sheetFormatPr defaultColWidth="34.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="56.7265625" style="23" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" style="23" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" style="23" customWidth="1"/>
-    <col min="4" max="20" width="42.7265625" style="23" customWidth="1"/>
-    <col min="21" max="16384" width="34.7265625" style="23"/>
+    <col min="1" max="1" width="56.7265625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="16.7265625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" style="16" customWidth="1"/>
+    <col min="4" max="20" width="42.7265625" style="16" customWidth="1"/>
+    <col min="21" max="16384" width="34.7265625" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="264" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="21"/>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="22"/>
-      <c r="R1" s="22"/>
-      <c r="S1" s="22"/>
+      <c r="A1" s="68"/>
+      <c r="B1" s="68"/>
+      <c r="C1" s="68"/>
+      <c r="D1" s="68"/>
+      <c r="E1" s="68"/>
+      <c r="F1" s="68"/>
+      <c r="G1" s="68"/>
+      <c r="H1" s="68"/>
+      <c r="I1" s="68"/>
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69" t="s">
+        <v>13</v>
+      </c>
+      <c r="S1" s="69"/>
+      <c r="T1" s="69"/>
     </row>
     <row r="2" spans="1:20" ht="190.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="75" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="75"/>
+      <c r="C2" s="75"/>
+      <c r="D2" s="75"/>
+      <c r="E2" s="75"/>
+      <c r="F2" s="75"/>
+      <c r="G2" s="75"/>
+      <c r="H2" s="75"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="75"/>
+      <c r="L2" s="75"/>
+      <c r="M2" s="75"/>
+      <c r="N2" s="75"/>
+      <c r="O2" s="75"/>
+      <c r="P2" s="75"/>
+      <c r="Q2" s="75"/>
+      <c r="R2" s="75"/>
+      <c r="S2" s="75"/>
+      <c r="T2" s="75"/>
+    </row>
+    <row r="3" spans="1:20" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="67"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71"/>
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
+      <c r="Q3" s="71"/>
+      <c r="R3" s="71"/>
+      <c r="S3" s="71"/>
+      <c r="T3" s="71"/>
+    </row>
+    <row r="4" spans="1:20" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="74"/>
-      <c r="J2" s="74"/>
-      <c r="K2" s="74"/>
-      <c r="L2" s="74"/>
-      <c r="M2" s="74"/>
-      <c r="N2" s="74"/>
-      <c r="O2" s="74"/>
-      <c r="P2" s="74"/>
-      <c r="Q2" s="74"/>
-      <c r="R2" s="74"/>
-      <c r="S2" s="74"/>
-      <c r="T2" s="74"/>
-    </row>
-    <row r="3" spans="1:20" ht="49.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="19"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-    </row>
-    <row r="4" spans="1:20" ht="76.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="75" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
-      <c r="M4" s="75"/>
-      <c r="N4" s="75"/>
-      <c r="O4" s="75"/>
-      <c r="P4" s="75"/>
-      <c r="Q4" s="75"/>
-      <c r="R4" s="75"/>
-      <c r="S4" s="75"/>
-      <c r="T4" s="75"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1773,51 +1725,51 @@
   <dimension ref="A1:W26"/>
   <sheetFormatPr defaultColWidth="34.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="56.7265625" style="23" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" style="23" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" style="23" customWidth="1"/>
-    <col min="4" max="20" width="42.7265625" style="23" customWidth="1"/>
-    <col min="21" max="16384" width="34.7265625" style="23"/>
+    <col min="1" max="1" width="56.7265625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="16.7265625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" style="16" customWidth="1"/>
+    <col min="4" max="20" width="42.7265625" style="16" customWidth="1"/>
+    <col min="21" max="16384" width="34.7265625" style="16"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="76" t="s">
+      <c r="B1" s="77" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="77"/>
+      <c r="C1" s="78"/>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E1" s="2"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="25"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="18"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="64"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="57"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="16"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="14"/>
       <c r="N1" s="1"/>
       <c r="O1" s="2"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="14"/>
-      <c r="R1" s="16"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="12"/>
+      <c r="R1" s="14"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
     </row>
-    <row r="2" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="78"/>
-      <c r="B2" s="81" t="s">
+    <row r="2" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="79"/>
+      <c r="B2" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="84" t="s">
+      <c r="C2" s="85" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="5"/>
-      <c r="E2" s="15"/>
+      <c r="E2" s="13"/>
       <c r="F2" s="5"/>
       <c r="G2" s="5"/>
       <c r="H2" s="5"/>
@@ -1828,84 +1780,84 @@
       <c r="M2" s="7"/>
       <c r="N2" s="5"/>
       <c r="O2" s="7"/>
-      <c r="P2" s="15"/>
+      <c r="P2" s="13"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="5"/>
       <c r="S2" s="7"/>
       <c r="T2" s="7"/>
     </row>
-    <row r="3" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="79"/>
-      <c r="B3" s="82"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33"/>
-      <c r="I3" s="33"/>
+    <row r="3" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="80"/>
+      <c r="B3" s="83"/>
+      <c r="C3" s="86"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="26"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="26"/>
+      <c r="I3" s="26"/>
       <c r="J3" s="8"/>
       <c r="K3" s="5"/>
       <c r="L3" s="5"/>
       <c r="M3" s="5"/>
-      <c r="N3" s="33"/>
+      <c r="N3" s="26"/>
       <c r="O3" s="5"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="36"/>
-      <c r="R3" s="33"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="26"/>
       <c r="S3" s="5"/>
       <c r="T3" s="5"/>
     </row>
-    <row r="4" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="79"/>
-      <c r="B4" s="82"/>
-      <c r="C4" s="85"/>
-      <c r="D4" s="35"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="35"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
-      <c r="I4" s="33"/>
-      <c r="J4" s="52"/>
-      <c r="K4" s="33"/>
-      <c r="L4" s="36"/>
-      <c r="M4" s="36"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="36"/>
-      <c r="P4" s="35"/>
-      <c r="Q4" s="35"/>
-      <c r="R4" s="35"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-    </row>
-    <row r="5" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="79"/>
-      <c r="B5" s="83"/>
-      <c r="C5" s="86"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="38"/>
-      <c r="O5" s="38"/>
-      <c r="P5" s="37"/>
-      <c r="Q5" s="39"/>
-      <c r="R5" s="37"/>
-      <c r="S5" s="38"/>
-      <c r="T5" s="38"/>
-    </row>
-    <row r="6" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="79"/>
-      <c r="B6" s="87" t="s">
+    <row r="4" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="80"/>
+      <c r="B4" s="83"/>
+      <c r="C4" s="86"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28"/>
+      <c r="I4" s="26"/>
+      <c r="J4" s="45"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="29"/>
+      <c r="M4" s="29"/>
+      <c r="N4" s="26"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="28"/>
+      <c r="Q4" s="28"/>
+      <c r="R4" s="28"/>
+      <c r="S4" s="29"/>
+      <c r="T4" s="29"/>
+    </row>
+    <row r="5" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="80"/>
+      <c r="B5" s="84"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="31"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="47"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
+      <c r="O5" s="31"/>
+      <c r="P5" s="30"/>
+      <c r="Q5" s="32"/>
+      <c r="R5" s="30"/>
+      <c r="S5" s="31"/>
+      <c r="T5" s="31"/>
+    </row>
+    <row r="6" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="80"/>
+      <c r="B6" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="88" t="s">
+      <c r="C6" s="89" t="s">
         <v>1</v>
       </c>
       <c r="D6" s="5"/>
@@ -1926,182 +1878,182 @@
       <c r="S6" s="5"/>
       <c r="T6" s="5"/>
     </row>
-    <row r="7" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="79"/>
-      <c r="B7" s="82"/>
-      <c r="C7" s="85"/>
-      <c r="D7" s="33"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="33"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="33"/>
+    <row r="7" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="80"/>
+      <c r="B7" s="83"/>
+      <c r="C7" s="86"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="26"/>
       <c r="I7" s="5"/>
       <c r="J7" s="8"/>
-      <c r="K7" s="33"/>
-      <c r="L7" s="33"/>
-      <c r="M7" s="33"/>
-      <c r="N7" s="33"/>
-      <c r="O7" s="33"/>
-      <c r="P7" s="33"/>
-      <c r="Q7" s="36"/>
-      <c r="R7" s="61"/>
-      <c r="S7" s="33"/>
-      <c r="T7" s="33"/>
-    </row>
-    <row r="8" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="79"/>
-      <c r="B8" s="82"/>
-      <c r="C8" s="85"/>
-      <c r="D8" s="35"/>
-      <c r="E8" s="35"/>
-      <c r="F8" s="35"/>
-      <c r="G8" s="35"/>
-      <c r="H8" s="35"/>
-      <c r="I8" s="35"/>
-      <c r="J8" s="52"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="35"/>
-      <c r="M8" s="35"/>
-      <c r="N8" s="35"/>
-      <c r="O8" s="35"/>
-      <c r="P8" s="35"/>
-      <c r="Q8" s="35"/>
-      <c r="R8" s="52"/>
-      <c r="S8" s="35"/>
-      <c r="T8" s="35"/>
-    </row>
-    <row r="9" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="79"/>
-      <c r="B9" s="83"/>
-      <c r="C9" s="85"/>
-      <c r="D9" s="60"/>
-      <c r="E9" s="53"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="54"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="37"/>
-      <c r="M9" s="37"/>
-      <c r="N9" s="38"/>
-      <c r="O9" s="37"/>
-      <c r="P9" s="38"/>
-      <c r="Q9" s="38"/>
-      <c r="R9" s="55"/>
-      <c r="S9" s="37"/>
-      <c r="T9" s="37"/>
-    </row>
-    <row r="10" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="79"/>
-      <c r="B10" s="89" t="s">
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="26"/>
+      <c r="O7" s="26"/>
+      <c r="P7" s="26"/>
+      <c r="Q7" s="29"/>
+      <c r="R7" s="54"/>
+      <c r="S7" s="26"/>
+      <c r="T7" s="26"/>
+    </row>
+    <row r="8" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="80"/>
+      <c r="B8" s="83"/>
+      <c r="C8" s="86"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="45"/>
+      <c r="K8" s="26"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
+      <c r="R8" s="45"/>
+      <c r="S8" s="28"/>
+      <c r="T8" s="28"/>
+    </row>
+    <row r="9" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="80"/>
+      <c r="B9" s="84"/>
+      <c r="C9" s="86"/>
+      <c r="D9" s="53"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="30"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="31"/>
+      <c r="O9" s="30"/>
+      <c r="P9" s="31"/>
+      <c r="Q9" s="31"/>
+      <c r="R9" s="48"/>
+      <c r="S9" s="30"/>
+      <c r="T9" s="30"/>
+    </row>
+    <row r="10" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="80"/>
+      <c r="B10" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="C10" s="92" t="s">
+      <c r="C10" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="63"/>
-      <c r="E10" s="56"/>
-      <c r="F10" s="40"/>
-      <c r="G10" s="41"/>
-      <c r="H10" s="62"/>
-      <c r="I10" s="42"/>
-      <c r="J10" s="65"/>
-      <c r="K10" s="28"/>
-      <c r="L10" s="26"/>
-      <c r="M10" s="26"/>
-      <c r="N10" s="27"/>
-      <c r="O10" s="26"/>
-      <c r="P10" s="41"/>
-      <c r="Q10" s="43"/>
-      <c r="R10" s="56"/>
-      <c r="S10" s="26"/>
-      <c r="T10" s="26"/>
+      <c r="D10" s="56"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="33"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="35"/>
+      <c r="J10" s="58"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="20"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="36"/>
+      <c r="R10" s="49"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
       <c r="U10" s="6"/>
       <c r="V10" s="6"/>
       <c r="W10" s="6"/>
     </row>
-    <row r="11" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="79"/>
-      <c r="B11" s="90"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="57"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="44"/>
-      <c r="G11" s="45"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="31"/>
-      <c r="J11" s="29"/>
-      <c r="K11" s="31"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="31"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="45"/>
-      <c r="Q11" s="46"/>
-      <c r="R11" s="47"/>
-      <c r="S11" s="30"/>
-      <c r="T11" s="30"/>
+    <row r="11" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="80"/>
+      <c r="B11" s="91"/>
+      <c r="C11" s="94"/>
+      <c r="D11" s="50"/>
+      <c r="E11" s="40"/>
+      <c r="F11" s="37"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="40"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="22"/>
+      <c r="K11" s="24"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="24"/>
+      <c r="O11" s="23"/>
+      <c r="P11" s="38"/>
+      <c r="Q11" s="39"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="23"/>
+      <c r="T11" s="23"/>
       <c r="U11" s="3"/>
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
     </row>
-    <row r="12" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="79"/>
-      <c r="B12" s="90"/>
-      <c r="C12" s="93"/>
-      <c r="D12" s="47"/>
-      <c r="E12" s="47"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="47"/>
-      <c r="H12" s="44"/>
-      <c r="I12" s="47"/>
-      <c r="J12" s="66"/>
-      <c r="K12" s="45"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="31"/>
-      <c r="O12" s="47"/>
-      <c r="P12" s="47"/>
-      <c r="Q12" s="45"/>
-      <c r="R12" s="45"/>
-      <c r="S12" s="47"/>
-      <c r="T12" s="47"/>
+    <row r="12" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="80"/>
+      <c r="B12" s="91"/>
+      <c r="C12" s="94"/>
+      <c r="D12" s="40"/>
+      <c r="E12" s="40"/>
+      <c r="F12" s="37"/>
+      <c r="G12" s="40"/>
+      <c r="H12" s="37"/>
+      <c r="I12" s="40"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="40"/>
+      <c r="M12" s="40"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="40"/>
+      <c r="Q12" s="38"/>
+      <c r="R12" s="38"/>
+      <c r="S12" s="40"/>
+      <c r="T12" s="40"/>
       <c r="U12" s="3"/>
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
     </row>
-    <row r="13" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="79"/>
-      <c r="B13" s="91"/>
-      <c r="C13" s="94"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="48"/>
-      <c r="H13" s="58"/>
-      <c r="I13" s="58"/>
-      <c r="J13" s="58"/>
-      <c r="K13" s="48"/>
-      <c r="L13" s="49"/>
-      <c r="M13" s="49"/>
-      <c r="N13" s="48"/>
-      <c r="O13" s="49"/>
-      <c r="P13" s="48"/>
-      <c r="Q13" s="48"/>
-      <c r="R13" s="48"/>
-      <c r="S13" s="49"/>
-      <c r="T13" s="49"/>
+    <row r="13" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="80"/>
+      <c r="B13" s="92"/>
+      <c r="C13" s="95"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="42"/>
+      <c r="G13" s="41"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="51"/>
+      <c r="K13" s="41"/>
+      <c r="L13" s="42"/>
+      <c r="M13" s="42"/>
+      <c r="N13" s="41"/>
+      <c r="O13" s="42"/>
+      <c r="P13" s="41"/>
+      <c r="Q13" s="41"/>
+      <c r="R13" s="41"/>
+      <c r="S13" s="42"/>
+      <c r="T13" s="42"/>
       <c r="U13" s="3"/>
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
     </row>
-    <row r="14" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="79"/>
-      <c r="B14" s="82" t="s">
+    <row r="14" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="80"/>
+      <c r="B14" s="83" t="s">
         <v>5</v>
       </c>
-      <c r="C14" s="95" t="s">
+      <c r="C14" s="96" t="s">
         <v>8</v>
       </c>
       <c r="D14" s="5"/>
@@ -2124,81 +2076,81 @@
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
     </row>
-    <row r="15" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="79"/>
-      <c r="B15" s="82"/>
-      <c r="C15" s="85"/>
-      <c r="D15" s="33"/>
-      <c r="E15" s="33"/>
-      <c r="F15" s="33"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
-      <c r="I15" s="33"/>
+    <row r="15" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="80"/>
+      <c r="B15" s="83"/>
+      <c r="C15" s="86"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
       <c r="J15" s="8"/>
-      <c r="K15" s="33"/>
-      <c r="L15" s="33"/>
-      <c r="M15" s="33"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
       <c r="N15" s="5"/>
-      <c r="O15" s="33"/>
-      <c r="P15" s="33"/>
-      <c r="Q15" s="33"/>
-      <c r="R15" s="33"/>
-      <c r="S15" s="51"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="26"/>
+      <c r="R15" s="26"/>
+      <c r="S15" s="44"/>
       <c r="T15" s="5"/>
       <c r="V15" s="3"/>
       <c r="W15" s="3"/>
     </row>
-    <row r="16" spans="1:23" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="79"/>
-      <c r="B16" s="82"/>
-      <c r="C16" s="85"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="52"/>
-      <c r="K16" s="33"/>
-      <c r="L16" s="52"/>
-      <c r="M16" s="52"/>
-      <c r="N16" s="52"/>
-      <c r="O16" s="52"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="35"/>
-      <c r="R16" s="52"/>
-      <c r="S16" s="52"/>
-      <c r="T16" s="33"/>
-    </row>
-    <row r="17" spans="1:20" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="79"/>
-      <c r="B17" s="83"/>
-      <c r="C17" s="86"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="55"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="38"/>
-      <c r="J17" s="54"/>
-      <c r="K17" s="38"/>
-      <c r="L17" s="54"/>
-      <c r="M17" s="54"/>
-      <c r="N17" s="38"/>
-      <c r="O17" s="54"/>
-      <c r="P17" s="38"/>
-      <c r="Q17" s="38"/>
-      <c r="R17" s="54"/>
-      <c r="S17" s="54"/>
-      <c r="T17" s="38"/>
-    </row>
-    <row r="18" spans="1:20" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="79"/>
-      <c r="B18" s="87" t="s">
+    <row r="16" spans="1:23" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="80"/>
+      <c r="B16" s="83"/>
+      <c r="C16" s="86"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="45"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="45"/>
+      <c r="M16" s="45"/>
+      <c r="N16" s="45"/>
+      <c r="O16" s="45"/>
+      <c r="P16" s="28"/>
+      <c r="Q16" s="28"/>
+      <c r="R16" s="45"/>
+      <c r="S16" s="45"/>
+      <c r="T16" s="26"/>
+    </row>
+    <row r="17" spans="1:20" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="80"/>
+      <c r="B17" s="84"/>
+      <c r="C17" s="87"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="47"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="47"/>
+      <c r="M17" s="47"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="47"/>
+      <c r="P17" s="31"/>
+      <c r="Q17" s="31"/>
+      <c r="R17" s="47"/>
+      <c r="S17" s="47"/>
+      <c r="T17" s="31"/>
+    </row>
+    <row r="18" spans="1:20" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="80"/>
+      <c r="B18" s="88" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="85" t="s">
-        <v>12</v>
+      <c r="C18" s="86" t="s">
+        <v>11</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
@@ -2218,93 +2170,93 @@
       <c r="S18" s="4"/>
       <c r="T18" s="4"/>
     </row>
-    <row r="19" spans="1:20" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="79"/>
-      <c r="B19" s="82"/>
-      <c r="C19" s="85"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
+    <row r="19" spans="1:20" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="80"/>
+      <c r="B19" s="83"/>
+      <c r="C19" s="86"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
       <c r="H19" s="5"/>
-      <c r="I19" s="51"/>
+      <c r="I19" s="44"/>
       <c r="J19" s="8"/>
-      <c r="K19" s="33"/>
+      <c r="K19" s="26"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="33"/>
+      <c r="N19" s="26"/>
       <c r="O19" s="5"/>
       <c r="P19" s="5"/>
       <c r="Q19" s="5"/>
-      <c r="R19" s="33"/>
+      <c r="R19" s="26"/>
       <c r="S19" s="5"/>
       <c r="T19" s="5"/>
     </row>
-    <row r="20" spans="1:20" s="24" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="79"/>
-      <c r="B20" s="82"/>
-      <c r="C20" s="85"/>
-      <c r="D20" s="33"/>
-      <c r="E20" s="35"/>
-      <c r="F20" s="35"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="51"/>
-      <c r="J20" s="52"/>
-      <c r="K20" s="33"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35"/>
-      <c r="N20" s="35"/>
-      <c r="O20" s="35"/>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="35"/>
-      <c r="R20" s="35"/>
-      <c r="S20" s="35"/>
-      <c r="T20" s="35"/>
-    </row>
-    <row r="21" spans="1:20" s="24" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A21" s="80"/>
-      <c r="B21" s="96"/>
-      <c r="C21" s="97"/>
-      <c r="D21" s="34"/>
-      <c r="E21" s="34"/>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="67"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="50"/>
-      <c r="M21" s="34"/>
-      <c r="N21" s="34"/>
-      <c r="O21" s="59"/>
-      <c r="P21" s="34"/>
-      <c r="Q21" s="34"/>
-      <c r="R21" s="34"/>
-      <c r="S21" s="34"/>
-      <c r="T21" s="50"/>
+    <row r="20" spans="1:20" s="17" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="80"/>
+      <c r="B20" s="83"/>
+      <c r="C20" s="86"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="44"/>
+      <c r="J20" s="45"/>
+      <c r="K20" s="26"/>
+      <c r="L20" s="28"/>
+      <c r="M20" s="28"/>
+      <c r="N20" s="28"/>
+      <c r="O20" s="28"/>
+      <c r="P20" s="28"/>
+      <c r="Q20" s="28"/>
+      <c r="R20" s="28"/>
+      <c r="S20" s="28"/>
+      <c r="T20" s="28"/>
+    </row>
+    <row r="21" spans="1:20" s="17" customFormat="1" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A21" s="81"/>
+      <c r="B21" s="97"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="60"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="43"/>
+      <c r="M21" s="27"/>
+      <c r="N21" s="27"/>
+      <c r="O21" s="52"/>
+      <c r="P21" s="27"/>
+      <c r="Q21" s="27"/>
+      <c r="R21" s="27"/>
+      <c r="S21" s="27"/>
+      <c r="T21" s="43"/>
     </row>
     <row r="22" spans="1:20" ht="33" x14ac:dyDescent="0.35">
-      <c r="A22" s="68"/>
-      <c r="B22" s="69"/>
-      <c r="C22" s="69"/>
+      <c r="A22" s="61"/>
+      <c r="B22" s="62"/>
+      <c r="C22" s="62"/>
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="70"/>
-      <c r="I22" s="71"/>
-      <c r="J22" s="71"/>
-      <c r="K22" s="71"/>
-      <c r="L22" s="71"/>
+      <c r="H22" s="63"/>
+      <c r="I22" s="64"/>
+      <c r="J22" s="64"/>
+      <c r="K22" s="64"/>
+      <c r="L22" s="64"/>
       <c r="M22" s="3"/>
       <c r="N22" s="3"/>
-      <c r="O22" s="72"/>
+      <c r="O22" s="65"/>
       <c r="P22" s="3"/>
-      <c r="Q22" s="69"/>
-      <c r="R22" s="69"/>
-      <c r="S22" s="69"/>
-      <c r="T22" s="73"/>
+      <c r="Q22" s="62"/>
+      <c r="R22" s="62"/>
+      <c r="S22" s="62"/>
+      <c r="T22" s="66"/>
     </row>
     <row r="23" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
       <c r="Q23" s="3"/>
@@ -2352,159 +2304,240 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
+  <dimension ref="A1:T15"/>
   <sheetFormatPr defaultColWidth="34.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="56.7265625" style="23" customWidth="1"/>
-    <col min="2" max="2" width="16.7265625" style="23" customWidth="1"/>
-    <col min="3" max="3" width="28.7265625" style="23" customWidth="1"/>
-    <col min="4" max="20" width="42.7265625" style="23" customWidth="1"/>
-    <col min="21" max="16384" width="34.7265625" style="23"/>
+    <col min="1" max="1" width="56.7265625" style="16" customWidth="1"/>
+    <col min="2" max="2" width="16.7265625" style="16" customWidth="1"/>
+    <col min="3" max="3" width="28.7265625" style="16" customWidth="1"/>
+    <col min="4" max="20" width="42.7265625" style="16" customWidth="1"/>
+    <col min="21" max="16384" width="34.7265625" style="16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="17" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B1" s="98"/>
+    <row r="1" spans="1:20" s="15" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="62"/>
+      <c r="B1" s="99"/>
       <c r="C1" s="99"/>
-      <c r="D1" s="6"/>
+      <c r="D1" s="3"/>
       <c r="E1" s="3"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
-      <c r="O1" s="18"/>
-      <c r="P1" s="18"/>
-      <c r="Q1" s="18"/>
-      <c r="R1" s="18"/>
-      <c r="S1" s="18"/>
-    </row>
-    <row r="2" spans="1:20" s="17" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="98"/>
-      <c r="C2" s="99"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="18"/>
-      <c r="L2" s="18"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="18"/>
-      <c r="O2" s="18"/>
-      <c r="P2" s="18"/>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="18"/>
-      <c r="S2" s="18"/>
-    </row>
-    <row r="3" spans="1:20" s="17" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10"/>
-      <c r="B3" s="98"/>
-      <c r="C3" s="99"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="11"/>
-      <c r="H3" s="11"/>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="S3" s="11"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="100"/>
+      <c r="J1" s="100"/>
+      <c r="K1" s="100"/>
+      <c r="L1" s="100"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="72"/>
+      <c r="R1" s="72"/>
+      <c r="S1" s="72"/>
+      <c r="T1" s="72"/>
+    </row>
+    <row r="2" spans="1:20" s="15" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="62"/>
+      <c r="B2" s="62"/>
+      <c r="C2" s="62"/>
+      <c r="D2" s="62"/>
+      <c r="E2" s="62"/>
+      <c r="F2" s="62"/>
+      <c r="G2" s="62"/>
+      <c r="H2" s="62"/>
+      <c r="I2" s="62"/>
+      <c r="J2" s="62"/>
+      <c r="K2" s="62"/>
+      <c r="L2" s="62"/>
+      <c r="M2" s="62"/>
+      <c r="N2" s="62"/>
+      <c r="O2" s="62"/>
+      <c r="P2" s="62"/>
+      <c r="Q2" s="62"/>
+      <c r="R2" s="62"/>
+      <c r="S2" s="62"/>
+      <c r="T2" s="62"/>
+    </row>
+    <row r="3" spans="1:20" s="15" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="62"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
+      <c r="D3" s="62"/>
+      <c r="E3" s="62"/>
+      <c r="F3" s="62"/>
+      <c r="G3" s="62"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
+      <c r="K3" s="62"/>
+      <c r="L3" s="62"/>
+      <c r="M3" s="62"/>
+      <c r="N3" s="62"/>
+      <c r="O3" s="62"/>
+      <c r="P3" s="62"/>
+      <c r="Q3" s="62"/>
+      <c r="R3" s="62"/>
+      <c r="S3" s="62"/>
+      <c r="T3" s="62"/>
     </row>
     <row r="4" spans="1:20" s="10" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="98"/>
-      <c r="C4" s="99"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="100"/>
-      <c r="I4" s="100"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
-      <c r="S4" s="11"/>
+      <c r="A4" s="62"/>
+      <c r="B4" s="62"/>
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="62"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="62"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="62"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="62"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="62"/>
+      <c r="P4" s="62"/>
+      <c r="Q4" s="62"/>
+      <c r="R4" s="62"/>
+      <c r="S4" s="62"/>
+      <c r="T4" s="62"/>
     </row>
     <row r="5" spans="1:20" s="10" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="17"/>
-      <c r="B5" s="98"/>
-      <c r="C5" s="99"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
-      <c r="K5" s="18"/>
-      <c r="L5" s="18"/>
-      <c r="M5" s="18"/>
-      <c r="N5" s="18"/>
-      <c r="O5" s="18"/>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
-      <c r="R5" s="18"/>
-      <c r="S5" s="18"/>
-    </row>
-    <row r="6" spans="1:20" s="17" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="98"/>
-      <c r="C6" s="99"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-    </row>
-    <row r="7" spans="1:20" s="17" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="98"/>
-      <c r="C7" s="99"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
-      <c r="M7" s="18"/>
-      <c r="N7" s="18"/>
-      <c r="O7" s="18"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18"/>
-    </row>
-    <row r="11" spans="1:20" ht="28" x14ac:dyDescent="0.35">
-      <c r="Q11" s="6"/>
-      <c r="R11" s="6"/>
-      <c r="T11" s="6"/>
+      <c r="A5" s="62"/>
+      <c r="B5" s="62"/>
+      <c r="C5" s="62"/>
+      <c r="D5" s="62"/>
+      <c r="E5" s="62"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="62"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="62"/>
+      <c r="J5" s="62"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="62"/>
+      <c r="M5" s="62"/>
+      <c r="N5" s="62"/>
+      <c r="O5" s="62"/>
+      <c r="P5" s="62"/>
+      <c r="Q5" s="62"/>
+      <c r="R5" s="62"/>
+      <c r="S5" s="62"/>
+      <c r="T5" s="62"/>
+    </row>
+    <row r="6" spans="1:20" s="15" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="74"/>
+      <c r="B6" s="74"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="74"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="74"/>
+      <c r="J6" s="74"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="74"/>
+      <c r="M6" s="74"/>
+      <c r="N6" s="74"/>
+      <c r="O6" s="74"/>
+      <c r="P6" s="74"/>
+      <c r="Q6" s="74"/>
+      <c r="R6" s="74"/>
+      <c r="S6" s="74"/>
+      <c r="T6" s="74"/>
+    </row>
+    <row r="7" spans="1:20" s="15" customFormat="1" ht="26.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="74"/>
+      <c r="B7" s="74"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="74"/>
+      <c r="E7" s="74"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="74"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="74"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="74"/>
+      <c r="O7" s="74"/>
+      <c r="P7" s="74"/>
+      <c r="Q7" s="74"/>
+      <c r="R7" s="74"/>
+      <c r="S7" s="74"/>
+      <c r="T7" s="74"/>
+    </row>
+    <row r="8" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A8" s="62"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="62"/>
+      <c r="K8" s="62"/>
+      <c r="L8" s="62"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="62"/>
+      <c r="O8" s="62"/>
+      <c r="P8" s="62"/>
+      <c r="Q8" s="62"/>
+      <c r="R8" s="62"/>
+      <c r="S8" s="62"/>
+      <c r="T8" s="62"/>
+    </row>
+    <row r="9" spans="1:20" ht="28" x14ac:dyDescent="0.35">
+      <c r="A9" s="62"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="62"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
+      <c r="L9" s="62"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="62"/>
+      <c r="O9" s="62"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="62"/>
+      <c r="R9" s="62"/>
+      <c r="S9" s="62"/>
+      <c r="T9" s="62"/>
+    </row>
+    <row r="10" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="A10" s="62"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="62"/>
+      <c r="E10" s="62"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="62"/>
+      <c r="K10" s="62"/>
+      <c r="L10" s="62"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="62"/>
+      <c r="O10" s="62"/>
+      <c r="P10" s="62"/>
+      <c r="Q10" s="62"/>
+      <c r="R10" s="62"/>
+      <c r="S10" s="62"/>
+      <c r="T10" s="62"/>
+    </row>
+    <row r="11" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
+      <c r="Q11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="T11" s="3"/>
     </row>
     <row r="12" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
       <c r="Q12" s="3"/>
@@ -2526,23 +2559,10 @@
       <c r="R15" s="3"/>
       <c r="T15" s="3"/>
     </row>
-    <row r="16" spans="1:20" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="Q16" s="3"/>
-      <c r="R16" s="3"/>
-      <c r="T16" s="3"/>
-    </row>
-    <row r="17" spans="17:20" ht="25.5" x14ac:dyDescent="0.35">
-      <c r="Q17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="T17" s="3"/>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="C4:C7"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
+  <mergeCells count="2">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="I1:L1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.41" bottom="0.15748031496062992" header="0" footer="0"/>

</xml_diff>